<commit_message>
data from azam sb
data from azam sb
</commit_message>
<xml_diff>
--- a/1stJuly26/Surveyv + Gpx.xlsx
+++ b/1stJuly26/Surveyv + Gpx.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\barqaab\1stJuly26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Barqaab\1stJuly26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3B29F75-A73E-48BA-9FBD-E11299A2E5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AD5733-D45A-4A62-9C53-968B8E89C085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HtSurveyForm - 081025" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,43 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Zahid</author>
+  </authors>
+  <commentList>
+    <comment ref="J2" authorId="0" shapeId="0" xr:uid="{1C610767-B052-4CF6-A1FE-D38DF81F8625}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Zahid:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+it is serveyer id also availabl in HT / LT form group column in HT
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="171">
   <si>
     <t>Data Form for HT (GIS Survey Barqaab - PPL - OMS Consortium)</t>
   </si>
@@ -602,12 +637,15 @@
   <si>
     <t>mcm</t>
   </si>
+  <si>
+    <t>01 to 22 code 0r may be 99: srvy nme</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -652,8 +690,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -699,6 +750,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -836,64 +893,52 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="22" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -905,10 +950,19 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -941,23 +995,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -968,22 +1013,22 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="22" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -995,6 +1040,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1003,17 +1060,17 @@
   <dxfs count="4">
     <dxf>
       <fill>
-        <patternFill patternType="none">
+        <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor theme="5" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1057,8 +1114,8 @@
     <tableColumn id="5" xr3:uid="{4FA198CF-4D4D-44EA-A491-F49379D2BCD1}" name="ns1:time"/>
     <tableColumn id="6" xr3:uid="{B1F4108A-6D57-49C8-90D3-25D515B1AF67}" name="lat" dataDxfId="3"/>
     <tableColumn id="7" xr3:uid="{CE245AC8-8C21-4EA5-B23A-1F35D783E23D}" name="lon" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{1326B8B3-B9E0-4E13-BF98-A7507529F45F}" name="ns1:ele" dataDxfId="0"/>
-    <tableColumn id="9" xr3:uid="{463E0653-41EB-47B4-8F01-5A0D7950006C}" name="ns1:time2" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{1326B8B3-B9E0-4E13-BF98-A7507529F45F}" name="ns1:ele" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{463E0653-41EB-47B4-8F01-5A0D7950006C}" name="ns1:time2" dataDxfId="0"/>
     <tableColumn id="10" xr3:uid="{0CF6D097-A896-4136-B4BF-FF61F6257024}" name="ns1:name"/>
     <tableColumn id="11" xr3:uid="{F9E10501-0EF5-44F0-93FE-39B8E85F3890}" name="ns1:sym"/>
   </tableColumns>
@@ -1368,318 +1425,318 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="21">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="73"/>
-      <c r="U1" s="73"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="73"/>
-      <c r="X1" s="73"/>
-      <c r="Y1" s="73"/>
-      <c r="Z1" s="73"/>
-      <c r="AA1" s="73"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="73"/>
-      <c r="AD1" s="73"/>
-      <c r="AE1" s="73"/>
-      <c r="AF1" s="73"/>
-      <c r="AG1" s="74"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
+      <c r="R1" s="33"/>
+      <c r="S1" s="33"/>
+      <c r="T1" s="33"/>
+      <c r="U1" s="33"/>
+      <c r="V1" s="33"/>
+      <c r="W1" s="33"/>
+      <c r="X1" s="33"/>
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="33"/>
+      <c r="AA1" s="33"/>
+      <c r="AB1" s="33"/>
+      <c r="AC1" s="33"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="33"/>
+      <c r="AF1" s="33"/>
+      <c r="AG1" s="34"/>
     </row>
     <row r="2" spans="1:33">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="33" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="34"/>
-      <c r="K2" s="58" t="s">
+      <c r="J2" s="28"/>
+      <c r="K2" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="31" t="s">
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="49" t="s">
+      <c r="P2" s="45"/>
+      <c r="Q2" s="46"/>
+      <c r="R2" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="S2" s="50"/>
-      <c r="T2" s="51"/>
+      <c r="S2" s="51"/>
+      <c r="T2" s="52"/>
       <c r="U2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="V2" s="65">
+      <c r="V2" s="63">
         <v>4812</v>
       </c>
-      <c r="W2" s="66"/>
-      <c r="X2" s="33" t="s">
+      <c r="W2" s="64"/>
+      <c r="X2" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="Y2" s="37"/>
-      <c r="Z2" s="37"/>
-      <c r="AA2" s="37"/>
-      <c r="AB2" s="37"/>
-      <c r="AC2" s="37"/>
-      <c r="AD2" s="37"/>
-      <c r="AE2" s="34"/>
-      <c r="AF2" s="38" t="s">
+      <c r="Y2" s="27"/>
+      <c r="Z2" s="27"/>
+      <c r="AA2" s="27"/>
+      <c r="AB2" s="27"/>
+      <c r="AC2" s="27"/>
+      <c r="AD2" s="27"/>
+      <c r="AE2" s="28"/>
+      <c r="AF2" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="AG2" s="39"/>
+      <c r="AG2" s="42"/>
     </row>
     <row r="3" spans="1:33">
       <c r="A3" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="75"/>
-      <c r="C3" s="36"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="37"/>
       <c r="D3" s="15"/>
       <c r="E3" s="43"/>
       <c r="F3" s="43"/>
       <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="H3" s="24"/>
       <c r="I3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="36"/>
-      <c r="K3" s="61" t="s">
+      <c r="J3" s="37"/>
+      <c r="K3" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="62"/>
-      <c r="M3" s="62"/>
-      <c r="N3" s="63"/>
-      <c r="O3" s="46" t="s">
+      <c r="L3" s="60"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="47"/>
-      <c r="Q3" s="48"/>
-      <c r="R3" s="52" t="s">
+      <c r="P3" s="48"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="53"/>
-      <c r="T3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="55"/>
       <c r="U3" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="V3" s="64">
+      <c r="V3" s="23">
         <v>48123</v>
       </c>
-      <c r="W3" s="44"/>
-      <c r="X3" s="52"/>
-      <c r="Y3" s="53"/>
-      <c r="Z3" s="53"/>
-      <c r="AA3" s="53"/>
-      <c r="AB3" s="53"/>
-      <c r="AC3" s="53"/>
-      <c r="AD3" s="53"/>
-      <c r="AE3" s="53"/>
-      <c r="AF3" s="53"/>
-      <c r="AG3" s="54"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="53"/>
+      <c r="Y3" s="54"/>
+      <c r="Z3" s="54"/>
+      <c r="AA3" s="54"/>
+      <c r="AB3" s="54"/>
+      <c r="AC3" s="54"/>
+      <c r="AD3" s="54"/>
+      <c r="AE3" s="54"/>
+      <c r="AF3" s="54"/>
+      <c r="AG3" s="55"/>
     </row>
     <row r="4" spans="1:33">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
-      <c r="L4" s="41"/>
-      <c r="M4" s="42"/>
-      <c r="N4" s="40" t="s">
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="42"/>
-      <c r="P4" s="55"/>
-      <c r="Q4" s="56"/>
-      <c r="R4" s="56"/>
-      <c r="S4" s="56"/>
-      <c r="T4" s="56"/>
-      <c r="U4" s="56"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="56"/>
-      <c r="X4" s="56"/>
-      <c r="Y4" s="56"/>
-      <c r="Z4" s="56"/>
-      <c r="AA4" s="56"/>
-      <c r="AB4" s="56"/>
-      <c r="AC4" s="56"/>
-      <c r="AD4" s="56"/>
-      <c r="AE4" s="56"/>
-      <c r="AF4" s="56"/>
-      <c r="AG4" s="57"/>
+      <c r="O4" s="40"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="30"/>
+      <c r="R4" s="30"/>
+      <c r="S4" s="30"/>
+      <c r="T4" s="30"/>
+      <c r="U4" s="30"/>
+      <c r="V4" s="30"/>
+      <c r="W4" s="30"/>
+      <c r="X4" s="30"/>
+      <c r="Y4" s="30"/>
+      <c r="Z4" s="30"/>
+      <c r="AA4" s="30"/>
+      <c r="AB4" s="30"/>
+      <c r="AC4" s="30"/>
+      <c r="AD4" s="30"/>
+      <c r="AE4" s="30"/>
+      <c r="AF4" s="30"/>
+      <c r="AG4" s="31"/>
     </row>
     <row r="5" spans="1:33">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="72" t="s">
         <v>165</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="28" t="s">
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="70"/>
+      <c r="G5" s="70"/>
+      <c r="H5" s="70"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="70"/>
+      <c r="K5" s="70"/>
+      <c r="L5" s="70"/>
+      <c r="M5" s="71"/>
+      <c r="N5" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="O5" s="28"/>
+      <c r="O5" s="75"/>
       <c r="P5" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="Q5" s="30" t="s">
+      <c r="Q5" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30" t="s">
+      <c r="R5" s="67"/>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67" t="s">
         <v>18</v>
       </c>
-      <c r="U5" s="30"/>
-      <c r="V5" s="30"/>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="30"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="30"/>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="30"/>
-      <c r="AF5" s="30"/>
-      <c r="AG5" s="21" t="s">
+      <c r="U5" s="67"/>
+      <c r="V5" s="67"/>
+      <c r="W5" s="67"/>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="67"/>
+      <c r="Z5" s="67"/>
+      <c r="AA5" s="67"/>
+      <c r="AB5" s="67"/>
+      <c r="AC5" s="67"/>
+      <c r="AD5" s="67"/>
+      <c r="AE5" s="67"/>
+      <c r="AF5" s="67"/>
+      <c r="AG5" s="66" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:33">
-      <c r="A6" s="77"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="21" t="s">
+      <c r="A6" s="73"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="20" t="s">
+      <c r="D6" s="66"/>
+      <c r="E6" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="23" t="s">
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="77"/>
+      <c r="J6" s="77"/>
+      <c r="K6" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="27" t="s">
+      <c r="L6" s="62"/>
+      <c r="M6" s="62"/>
+      <c r="N6" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="O6" s="29" t="s">
+      <c r="O6" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="22" t="s">
+      <c r="P6" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="23" t="s">
+      <c r="Q6" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="R6" s="23" t="s">
+      <c r="R6" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="S6" s="23" t="s">
+      <c r="S6" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="T6" s="27" t="s">
+      <c r="T6" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="U6" s="27" t="s">
+      <c r="U6" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="V6" s="27" t="s">
+      <c r="V6" s="68" t="s">
         <v>44</v>
       </c>
-      <c r="W6" s="22" t="s">
+      <c r="W6" s="25" t="s">
         <v>19</v>
       </c>
       <c r="X6" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="Y6" s="22" t="s">
+      <c r="Y6" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="Z6" s="22" t="s">
+      <c r="Z6" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="AA6" s="27" t="s">
+      <c r="AA6" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="AB6" s="22" t="s">
+      <c r="AB6" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="AC6" s="22" t="s">
+      <c r="AC6" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="AD6" s="22" t="s">
+      <c r="AD6" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="AE6" s="27" t="s">
+      <c r="AE6" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="AF6" s="27" t="s">
+      <c r="AF6" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="AG6" s="21"/>
+      <c r="AG6" s="66"/>
     </row>
     <row r="7" spans="1:33" ht="20" customHeight="1">
-      <c r="A7" s="78"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
+      <c r="A7" s="74"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
       <c r="E7" s="17" t="s">
         <v>7</v>
       </c>
@@ -1698,31 +1755,31 @@
       <c r="J7" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="23"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="23"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
+      <c r="K7" s="62"/>
+      <c r="L7" s="62"/>
+      <c r="M7" s="62"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="62"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="62"/>
+      <c r="R7" s="62"/>
+      <c r="S7" s="62"/>
+      <c r="T7" s="25"/>
+      <c r="U7" s="25"/>
+      <c r="V7" s="25"/>
+      <c r="W7" s="25"/>
       <c r="X7" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="Y7" s="22"/>
-      <c r="Z7" s="22"/>
-      <c r="AA7" s="22"/>
-      <c r="AB7" s="22"/>
-      <c r="AC7" s="22"/>
-      <c r="AD7" s="22"/>
-      <c r="AE7" s="22"/>
-      <c r="AF7" s="22"/>
-      <c r="AG7" s="21"/>
+      <c r="Y7" s="25"/>
+      <c r="Z7" s="25"/>
+      <c r="AA7" s="25"/>
+      <c r="AB7" s="25"/>
+      <c r="AC7" s="25"/>
+      <c r="AD7" s="25"/>
+      <c r="AE7" s="25"/>
+      <c r="AF7" s="25"/>
+      <c r="AG7" s="66"/>
     </row>
     <row r="8" spans="1:33">
       <c r="A8" s="1">
@@ -1731,7 +1788,7 @@
       <c r="B8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="22">
         <v>0</v>
       </c>
       <c r="D8" s="1">
@@ -1799,12 +1856,14 @@
       <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="C9" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2">
@@ -2563,6 +2622,41 @@
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="AF6:AF7"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="P6:P7"/>
+    <mergeCell ref="Q6:Q7"/>
+    <mergeCell ref="R6:R7"/>
+    <mergeCell ref="S6:S7"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="V6:V7"/>
+    <mergeCell ref="C5:M5"/>
+    <mergeCell ref="AD6:AD7"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="AE6:AE7"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="C6:D7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="K6:M7"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="X3:AG3"/>
+    <mergeCell ref="AG5:AG7"/>
+    <mergeCell ref="T5:AF5"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="Y6:Y7"/>
+    <mergeCell ref="Z6:Z7"/>
+    <mergeCell ref="AA6:AA7"/>
+    <mergeCell ref="AB6:AB7"/>
+    <mergeCell ref="AC6:AC7"/>
+    <mergeCell ref="T6:T7"/>
+    <mergeCell ref="U6:U7"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="W6:W7"/>
     <mergeCell ref="X2:AE2"/>
     <mergeCell ref="P4:AG4"/>
     <mergeCell ref="A1:AG1"/>
@@ -2577,41 +2671,6 @@
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="K2:N2"/>
     <mergeCell ref="K3:N3"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="V3:W3"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="X3:AG3"/>
-    <mergeCell ref="AG5:AG7"/>
-    <mergeCell ref="T5:AF5"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="Y6:Y7"/>
-    <mergeCell ref="Z6:Z7"/>
-    <mergeCell ref="AA6:AA7"/>
-    <mergeCell ref="AB6:AB7"/>
-    <mergeCell ref="AC6:AC7"/>
-    <mergeCell ref="T6:T7"/>
-    <mergeCell ref="U6:U7"/>
-    <mergeCell ref="V6:V7"/>
-    <mergeCell ref="W6:W7"/>
-    <mergeCell ref="AD6:AD7"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="AE6:AE7"/>
-    <mergeCell ref="AF6:AF7"/>
-    <mergeCell ref="N5:O5"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="P6:P7"/>
-    <mergeCell ref="Q6:Q7"/>
-    <mergeCell ref="R6:R7"/>
-    <mergeCell ref="S6:S7"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="K6:M7"/>
-    <mergeCell ref="C5:M5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -2619,7 +2678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA80F6E5-4549-4ACD-B4F1-E6F5B68EB513}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA80F6E5-4549-4ACD-B4F1-E6F5B68EB513}">
   <dimension ref="A1:K93"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -2629,8 +2688,8 @@
     <col min="4" max="4" width="19.36328125" customWidth="1"/>
     <col min="5" max="5" width="19.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.81640625" style="69" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.26953125" style="69" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.26953125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.26953125" customWidth="1"/>
     <col min="11" max="11" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2657,10 +2716,10 @@
       <c r="G1" t="s">
         <v>153</v>
       </c>
-      <c r="H1" s="69" t="s">
+      <c r="H1" t="s">
         <v>152</v>
       </c>
-      <c r="I1" s="70" t="s">
+      <c r="I1" s="20" t="s">
         <v>151</v>
       </c>
       <c r="J1" t="s">
@@ -2692,10 +2751,10 @@
       <c r="G2" s="9">
         <v>66.962320000000005</v>
       </c>
-      <c r="H2" s="69">
+      <c r="H2">
         <v>1610.357422</v>
       </c>
-      <c r="I2" s="71" t="s">
+      <c r="I2" s="21" t="s">
         <v>55</v>
       </c>
       <c r="J2" s="8" t="s">
@@ -2727,10 +2786,10 @@
       <c r="G3" s="9">
         <v>66.961999000000006</v>
       </c>
-      <c r="H3" s="69">
+      <c r="H3">
         <v>1608.9866939999999</v>
       </c>
-      <c r="I3" s="71" t="s">
+      <c r="I3" s="21" t="s">
         <v>148</v>
       </c>
       <c r="J3">
@@ -2762,10 +2821,10 @@
       <c r="G4" s="9">
         <v>66.961742999999998</v>
       </c>
-      <c r="H4" s="69">
+      <c r="H4">
         <v>1607.4956050000001</v>
       </c>
-      <c r="I4" s="71" t="s">
+      <c r="I4" s="21" t="s">
         <v>147</v>
       </c>
       <c r="J4">
@@ -2797,10 +2856,10 @@
       <c r="G5" s="9">
         <v>66.961447000000007</v>
       </c>
-      <c r="H5" s="69">
+      <c r="H5">
         <v>1607.4171140000001</v>
       </c>
-      <c r="I5" s="71" t="s">
+      <c r="I5" s="21" t="s">
         <v>146</v>
       </c>
       <c r="J5">
@@ -2832,10 +2891,10 @@
       <c r="G6" s="9">
         <v>66.961100999999999</v>
       </c>
-      <c r="H6" s="69">
+      <c r="H6">
         <v>1606.4837649999999</v>
       </c>
-      <c r="I6" s="71" t="s">
+      <c r="I6" s="21" t="s">
         <v>145</v>
       </c>
       <c r="J6">
@@ -2867,10 +2926,10 @@
       <c r="G7" s="9">
         <v>66.960700000000003</v>
       </c>
-      <c r="H7" s="69">
+      <c r="H7">
         <v>1607.252563</v>
       </c>
-      <c r="I7" s="71" t="s">
+      <c r="I7" s="21" t="s">
         <v>144</v>
       </c>
       <c r="J7">
@@ -2902,10 +2961,10 @@
       <c r="G8" s="9">
         <v>66.960203000000007</v>
       </c>
-      <c r="H8" s="69">
+      <c r="H8">
         <v>1603.856689</v>
       </c>
-      <c r="I8" s="71" t="s">
+      <c r="I8" s="21" t="s">
         <v>143</v>
       </c>
       <c r="J8">
@@ -2937,10 +2996,10 @@
       <c r="G9" s="9">
         <v>66.959749000000002</v>
       </c>
-      <c r="H9" s="69">
+      <c r="H9">
         <v>1606.4822999999999</v>
       </c>
-      <c r="I9" s="71" t="s">
+      <c r="I9" s="21" t="s">
         <v>142</v>
       </c>
       <c r="J9">
@@ -2972,10 +3031,10 @@
       <c r="G10" s="9">
         <v>66.959165999999996</v>
       </c>
-      <c r="H10" s="69">
+      <c r="H10">
         <v>1606.7120359999999</v>
       </c>
-      <c r="I10" s="71" t="s">
+      <c r="I10" s="21" t="s">
         <v>141</v>
       </c>
       <c r="J10">
@@ -3007,10 +3066,10 @@
       <c r="G11" s="9">
         <v>66.958926000000005</v>
       </c>
-      <c r="H11" s="69">
+      <c r="H11">
         <v>1607.0147710000001</v>
       </c>
-      <c r="I11" s="71" t="s">
+      <c r="I11" s="21" t="s">
         <v>140</v>
       </c>
       <c r="J11">
@@ -3042,10 +3101,10 @@
       <c r="G12" s="9">
         <v>66.958247</v>
       </c>
-      <c r="H12" s="69">
+      <c r="H12">
         <v>1607.0063479999999</v>
       </c>
-      <c r="I12" s="71" t="s">
+      <c r="I12" s="21" t="s">
         <v>139</v>
       </c>
       <c r="J12">
@@ -3077,10 +3136,10 @@
       <c r="G13" s="9">
         <v>66.957519000000005</v>
       </c>
-      <c r="H13" s="69">
+      <c r="H13">
         <v>1606.830933</v>
       </c>
-      <c r="I13" s="71" t="s">
+      <c r="I13" s="21" t="s">
         <v>138</v>
       </c>
       <c r="J13">
@@ -3112,10 +3171,10 @@
       <c r="G14" s="9">
         <v>66.956783999999999</v>
       </c>
-      <c r="H14" s="69">
+      <c r="H14">
         <v>1605.7977289999999</v>
       </c>
-      <c r="I14" s="71" t="s">
+      <c r="I14" s="21" t="s">
         <v>137</v>
       </c>
       <c r="J14">
@@ -3147,10 +3206,10 @@
       <c r="G15" s="9">
         <v>66.956256999999994</v>
       </c>
-      <c r="H15" s="69">
+      <c r="H15">
         <v>1605.966797</v>
       </c>
-      <c r="I15" s="71" t="s">
+      <c r="I15" s="21" t="s">
         <v>136</v>
       </c>
       <c r="J15">
@@ -3182,10 +3241,10 @@
       <c r="G16" s="9">
         <v>66.955875000000006</v>
       </c>
-      <c r="H16" s="69">
+      <c r="H16">
         <v>1605.6521</v>
       </c>
-      <c r="I16" s="71" t="s">
+      <c r="I16" s="21" t="s">
         <v>135</v>
       </c>
       <c r="J16">
@@ -3217,10 +3276,10 @@
       <c r="G17" s="9">
         <v>66.955357000000006</v>
       </c>
-      <c r="H17" s="69">
+      <c r="H17">
         <v>1605.6070560000001</v>
       </c>
-      <c r="I17" s="71" t="s">
+      <c r="I17" s="21" t="s">
         <v>134</v>
       </c>
       <c r="J17">
@@ -3252,10 +3311,10 @@
       <c r="G18" s="9">
         <v>66.954657999999995</v>
       </c>
-      <c r="H18" s="69">
+      <c r="H18">
         <v>1605.134033</v>
       </c>
-      <c r="I18" s="71" t="s">
+      <c r="I18" s="21" t="s">
         <v>133</v>
       </c>
       <c r="J18">
@@ -3287,10 +3346,10 @@
       <c r="G19" s="9">
         <v>66.953913999999997</v>
       </c>
-      <c r="H19" s="69">
+      <c r="H19">
         <v>1604.73938</v>
       </c>
-      <c r="I19" s="71" t="s">
+      <c r="I19" s="21" t="s">
         <v>132</v>
       </c>
       <c r="J19">
@@ -3322,10 +3381,10 @@
       <c r="G20" s="9">
         <v>66.953247000000005</v>
       </c>
-      <c r="H20" s="69">
+      <c r="H20">
         <v>1605.466919</v>
       </c>
-      <c r="I20" s="71" t="s">
+      <c r="I20" s="21" t="s">
         <v>131</v>
       </c>
       <c r="J20">
@@ -3357,10 +3416,10 @@
       <c r="G21" s="9">
         <v>66.952477999999999</v>
       </c>
-      <c r="H21" s="69">
+      <c r="H21">
         <v>1604.733154</v>
       </c>
-      <c r="I21" s="71" t="s">
+      <c r="I21" s="21" t="s">
         <v>130</v>
       </c>
       <c r="J21">
@@ -3392,10 +3451,10 @@
       <c r="G22" s="9">
         <v>66.951598000000004</v>
       </c>
-      <c r="H22" s="69">
+      <c r="H22">
         <v>1605.0325929999999</v>
       </c>
-      <c r="I22" s="71" t="s">
+      <c r="I22" s="21" t="s">
         <v>129</v>
       </c>
       <c r="J22">
@@ -3427,10 +3486,10 @@
       <c r="G23" s="9">
         <v>66.951006000000007</v>
       </c>
-      <c r="H23" s="69">
+      <c r="H23">
         <v>1604.0701899999999</v>
       </c>
-      <c r="I23" s="71" t="s">
+      <c r="I23" s="21" t="s">
         <v>128</v>
       </c>
       <c r="J23">
@@ -3462,10 +3521,10 @@
       <c r="G24" s="9">
         <v>66.950706999999994</v>
       </c>
-      <c r="H24" s="69">
+      <c r="H24">
         <v>1603.5732419999999</v>
       </c>
-      <c r="I24" s="71" t="s">
+      <c r="I24" s="21" t="s">
         <v>127</v>
       </c>
       <c r="J24">
@@ -3497,10 +3556,10 @@
       <c r="G25" s="9">
         <v>66.950333000000001</v>
       </c>
-      <c r="H25" s="69">
+      <c r="H25">
         <v>1602.951294</v>
       </c>
-      <c r="I25" s="71" t="s">
+      <c r="I25" s="21" t="s">
         <v>126</v>
       </c>
       <c r="J25">
@@ -3532,10 +3591,10 @@
       <c r="G26" s="9">
         <v>66.949793</v>
       </c>
-      <c r="H26" s="69">
+      <c r="H26">
         <v>1602.961548</v>
       </c>
-      <c r="I26" s="71" t="s">
+      <c r="I26" s="21" t="s">
         <v>125</v>
       </c>
       <c r="J26">
@@ -3567,10 +3626,10 @@
       <c r="G27" s="9">
         <v>66.949214999999995</v>
       </c>
-      <c r="H27" s="69">
+      <c r="H27">
         <v>1602.255005</v>
       </c>
-      <c r="I27" s="71" t="s">
+      <c r="I27" s="21" t="s">
         <v>124</v>
       </c>
       <c r="J27">
@@ -3602,10 +3661,10 @@
       <c r="G28" s="9">
         <v>66.948749000000007</v>
       </c>
-      <c r="H28" s="69">
+      <c r="H28">
         <v>1602.1285399999999</v>
       </c>
-      <c r="I28" s="71" t="s">
+      <c r="I28" s="21" t="s">
         <v>123</v>
       </c>
       <c r="J28">
@@ -3637,10 +3696,10 @@
       <c r="G29" s="9">
         <v>66.948626000000004</v>
       </c>
-      <c r="H29" s="69">
+      <c r="H29">
         <v>1601.650879</v>
       </c>
-      <c r="I29" s="71" t="s">
+      <c r="I29" s="21" t="s">
         <v>122</v>
       </c>
       <c r="J29">
@@ -3672,10 +3731,10 @@
       <c r="G30" s="9">
         <v>66.948026999999996</v>
       </c>
-      <c r="H30" s="69">
+      <c r="H30">
         <v>1602.0195309999999</v>
       </c>
-      <c r="I30" s="71" t="s">
+      <c r="I30" s="21" t="s">
         <v>121</v>
       </c>
       <c r="J30">
@@ -3707,10 +3766,10 @@
       <c r="G31" s="9">
         <v>66.947389999999999</v>
       </c>
-      <c r="H31" s="69">
+      <c r="H31">
         <v>1600.184937</v>
       </c>
-      <c r="I31" s="71" t="s">
+      <c r="I31" s="21" t="s">
         <v>120</v>
       </c>
       <c r="J31">
@@ -3742,10 +3801,10 @@
       <c r="G32" s="9">
         <v>66.946776999999997</v>
       </c>
-      <c r="H32" s="69">
+      <c r="H32">
         <v>1598.9360349999999</v>
       </c>
-      <c r="I32" s="71" t="s">
+      <c r="I32" s="21" t="s">
         <v>119</v>
       </c>
       <c r="J32">
@@ -3777,10 +3836,10 @@
       <c r="G33" s="9">
         <v>66.946121000000005</v>
       </c>
-      <c r="H33" s="69">
+      <c r="H33">
         <v>1597.957764</v>
       </c>
-      <c r="I33" s="71" t="s">
+      <c r="I33" s="21" t="s">
         <v>118</v>
       </c>
       <c r="J33">
@@ -3812,10 +3871,10 @@
       <c r="G34" s="9">
         <v>66.945627000000002</v>
       </c>
-      <c r="H34" s="69">
+      <c r="H34">
         <v>1597.605591</v>
       </c>
-      <c r="I34" s="71" t="s">
+      <c r="I34" s="21" t="s">
         <v>117</v>
       </c>
       <c r="J34">
@@ -3847,10 +3906,10 @@
       <c r="G35" s="9">
         <v>66.945100999999994</v>
       </c>
-      <c r="H35" s="69">
+      <c r="H35">
         <v>1596.5512699999999</v>
       </c>
-      <c r="I35" s="71" t="s">
+      <c r="I35" s="21" t="s">
         <v>116</v>
       </c>
       <c r="J35">
@@ -3882,10 +3941,10 @@
       <c r="G36" s="9">
         <v>66.945323999999999</v>
       </c>
-      <c r="H36" s="69">
+      <c r="H36">
         <v>1597.4576420000001</v>
       </c>
-      <c r="I36" s="71" t="s">
+      <c r="I36" s="21" t="s">
         <v>115</v>
       </c>
       <c r="J36">
@@ -3917,10 +3976,10 @@
       <c r="G37" s="9">
         <v>66.945851000000005</v>
       </c>
-      <c r="H37" s="69">
+      <c r="H37">
         <v>1598.317871</v>
       </c>
-      <c r="I37" s="71" t="s">
+      <c r="I37" s="21" t="s">
         <v>114</v>
       </c>
       <c r="J37">
@@ -3952,10 +4011,10 @@
       <c r="G38" s="9">
         <v>66.945846000000003</v>
       </c>
-      <c r="H38" s="69">
+      <c r="H38">
         <v>1598.2729489999999</v>
       </c>
-      <c r="I38" s="71" t="s">
+      <c r="I38" s="21" t="s">
         <v>113</v>
       </c>
       <c r="J38">
@@ -3987,10 +4046,10 @@
       <c r="G39" s="9">
         <v>66.944494000000006</v>
       </c>
-      <c r="H39" s="69">
+      <c r="H39">
         <v>1596.725342</v>
       </c>
-      <c r="I39" s="71" t="s">
+      <c r="I39" s="21" t="s">
         <v>112</v>
       </c>
       <c r="J39">
@@ -4022,10 +4081,10 @@
       <c r="G40" s="9">
         <v>66.944491999999997</v>
       </c>
-      <c r="H40" s="69">
+      <c r="H40">
         <v>1595.989746</v>
       </c>
-      <c r="I40" s="71" t="s">
+      <c r="I40" s="21" t="s">
         <v>111</v>
       </c>
       <c r="J40">
@@ -4057,10 +4116,10 @@
       <c r="G41" s="9">
         <v>66.943978999999999</v>
       </c>
-      <c r="H41" s="69">
+      <c r="H41">
         <v>1595.6669919999999</v>
       </c>
-      <c r="I41" s="71" t="s">
+      <c r="I41" s="21" t="s">
         <v>110</v>
       </c>
       <c r="J41">
@@ -4092,10 +4151,10 @@
       <c r="G42" s="9">
         <v>66.944103999999996</v>
       </c>
-      <c r="H42" s="69">
+      <c r="H42">
         <v>1595.3145750000001</v>
       </c>
-      <c r="I42" s="71" t="s">
+      <c r="I42" s="21" t="s">
         <v>109</v>
       </c>
       <c r="J42">
@@ -4127,10 +4186,10 @@
       <c r="G43" s="9">
         <v>66.944157000000004</v>
       </c>
-      <c r="H43" s="69">
+      <c r="H43">
         <v>1594.9195560000001</v>
       </c>
-      <c r="I43" s="71" t="s">
+      <c r="I43" s="21" t="s">
         <v>108</v>
       </c>
       <c r="J43">
@@ -4162,10 +4221,10 @@
       <c r="G44" s="9">
         <v>66.943906999999996</v>
       </c>
-      <c r="H44" s="69">
+      <c r="H44">
         <v>1595.8107910000001</v>
       </c>
-      <c r="I44" s="71" t="s">
+      <c r="I44" s="21" t="s">
         <v>107</v>
       </c>
       <c r="J44">
@@ -4197,10 +4256,10 @@
       <c r="G45" s="9">
         <v>66.943904000000003</v>
       </c>
-      <c r="H45" s="69">
+      <c r="H45">
         <v>1595.9229740000001</v>
       </c>
-      <c r="I45" s="71" t="s">
+      <c r="I45" s="21" t="s">
         <v>106</v>
       </c>
       <c r="J45">
@@ -4232,10 +4291,10 @@
       <c r="G46" s="9">
         <v>66.943859000000003</v>
       </c>
-      <c r="H46" s="69">
+      <c r="H46">
         <v>1595.7532960000001</v>
       </c>
-      <c r="I46" s="71" t="s">
+      <c r="I46" s="21" t="s">
         <v>105</v>
       </c>
       <c r="J46">
@@ -4267,10 +4326,10 @@
       <c r="G47" s="9">
         <v>66.943417999999994</v>
       </c>
-      <c r="H47" s="69">
+      <c r="H47">
         <v>1596.9564210000001</v>
       </c>
-      <c r="I47" s="71" t="s">
+      <c r="I47" s="21" t="s">
         <v>104</v>
       </c>
       <c r="J47">
@@ -4302,10 +4361,10 @@
       <c r="G48" s="9">
         <v>66.942898</v>
       </c>
-      <c r="H48" s="69">
+      <c r="H48">
         <v>1596.6561280000001</v>
       </c>
-      <c r="I48" s="71" t="s">
+      <c r="I48" s="21" t="s">
         <v>103</v>
       </c>
       <c r="J48">
@@ -4337,10 +4396,10 @@
       <c r="G49" s="9">
         <v>66.942339000000004</v>
       </c>
-      <c r="H49" s="69">
+      <c r="H49">
         <v>1596.077393</v>
       </c>
-      <c r="I49" s="71" t="s">
+      <c r="I49" s="21" t="s">
         <v>102</v>
       </c>
       <c r="J49">
@@ -4372,10 +4431,10 @@
       <c r="G50" s="9">
         <v>66.942313999999996</v>
       </c>
-      <c r="H50" s="69">
+      <c r="H50">
         <v>1596.3861079999999</v>
       </c>
-      <c r="I50" s="71" t="s">
+      <c r="I50" s="21" t="s">
         <v>101</v>
       </c>
       <c r="J50">
@@ -4407,10 +4466,10 @@
       <c r="G51" s="9">
         <v>66.942289000000002</v>
       </c>
-      <c r="H51" s="69">
+      <c r="H51">
         <v>1596.382202</v>
       </c>
-      <c r="I51" s="71" t="s">
+      <c r="I51" s="21" t="s">
         <v>100</v>
       </c>
       <c r="J51">
@@ -4442,10 +4501,10 @@
       <c r="G52" s="9">
         <v>66.941727999999998</v>
       </c>
-      <c r="H52" s="69">
+      <c r="H52">
         <v>1596.1479489999999</v>
       </c>
-      <c r="I52" s="71" t="s">
+      <c r="I52" s="21" t="s">
         <v>99</v>
       </c>
       <c r="J52">
@@ -4477,10 +4536,10 @@
       <c r="G53" s="9">
         <v>66.941231000000002</v>
       </c>
-      <c r="H53" s="69">
+      <c r="H53">
         <v>1595.8039550000001</v>
       </c>
-      <c r="I53" s="71" t="s">
+      <c r="I53" s="21" t="s">
         <v>98</v>
       </c>
       <c r="J53">
@@ -4512,10 +4571,10 @@
       <c r="G54" s="9">
         <v>66.941229000000007</v>
       </c>
-      <c r="H54" s="69">
+      <c r="H54">
         <v>1596.2574460000001</v>
       </c>
-      <c r="I54" s="71" t="s">
+      <c r="I54" s="21" t="s">
         <v>97</v>
       </c>
       <c r="J54">
@@ -4547,10 +4606,10 @@
       <c r="G55" s="9">
         <v>66.941222999999994</v>
       </c>
-      <c r="H55" s="69">
+      <c r="H55">
         <v>1596.24585</v>
       </c>
-      <c r="I55" s="71" t="s">
+      <c r="I55" s="21" t="s">
         <v>96</v>
       </c>
       <c r="J55">
@@ -4582,10 +4641,10 @@
       <c r="G56" s="9">
         <v>66.941204999999997</v>
       </c>
-      <c r="H56" s="69">
+      <c r="H56">
         <v>1596.2326660000001</v>
       </c>
-      <c r="I56" s="71" t="s">
+      <c r="I56" s="21" t="s">
         <v>95</v>
       </c>
       <c r="J56">
@@ -4617,10 +4676,10 @@
       <c r="G57" s="9">
         <v>66.940680999999998</v>
       </c>
-      <c r="H57" s="69">
+      <c r="H57">
         <v>1595.9520259999999</v>
       </c>
-      <c r="I57" s="71" t="s">
+      <c r="I57" s="21" t="s">
         <v>94</v>
       </c>
       <c r="J57">
@@ -4652,10 +4711,10 @@
       <c r="G58" s="9">
         <v>66.940136999999993</v>
       </c>
-      <c r="H58" s="69">
+      <c r="H58">
         <v>1595.7110600000001</v>
       </c>
-      <c r="I58" s="71" t="s">
+      <c r="I58" s="21" t="s">
         <v>93</v>
       </c>
       <c r="J58">
@@ -4687,10 +4746,10 @@
       <c r="G59" s="9">
         <v>66.939633000000001</v>
       </c>
-      <c r="H59" s="69">
+      <c r="H59">
         <v>1595.11438</v>
       </c>
-      <c r="I59" s="71" t="s">
+      <c r="I59" s="21" t="s">
         <v>92</v>
       </c>
       <c r="J59">
@@ -4722,10 +4781,10 @@
       <c r="G60" s="9">
         <v>66.939781999999994</v>
       </c>
-      <c r="H60" s="69">
+      <c r="H60">
         <v>1595.2150879999999</v>
       </c>
-      <c r="I60" s="71" t="s">
+      <c r="I60" s="21" t="s">
         <v>91</v>
       </c>
       <c r="J60">
@@ -4757,10 +4816,10 @@
       <c r="G61" s="9">
         <v>66.939763999999997</v>
       </c>
-      <c r="H61" s="69">
+      <c r="H61">
         <v>1595.190063</v>
       </c>
-      <c r="I61" s="71" t="s">
+      <c r="I61" s="21" t="s">
         <v>90</v>
       </c>
       <c r="J61">
@@ -4792,10 +4851,10 @@
       <c r="G62" s="9">
         <v>66.939942000000002</v>
       </c>
-      <c r="H62" s="69">
+      <c r="H62">
         <v>1594.1982419999999</v>
       </c>
-      <c r="I62" s="71" t="s">
+      <c r="I62" s="21" t="s">
         <v>89</v>
       </c>
       <c r="J62">
@@ -4827,10 +4886,10 @@
       <c r="G63" s="9">
         <v>66.940042000000005</v>
       </c>
-      <c r="H63" s="69">
+      <c r="H63">
         <v>1594.318237</v>
       </c>
-      <c r="I63" s="71" t="s">
+      <c r="I63" s="21" t="s">
         <v>88</v>
       </c>
       <c r="J63">
@@ -4862,10 +4921,10 @@
       <c r="G64" s="9">
         <v>66.940044999999998</v>
       </c>
-      <c r="H64" s="69">
+      <c r="H64">
         <v>1594.3054199999999</v>
       </c>
-      <c r="I64" s="71" t="s">
+      <c r="I64" s="21" t="s">
         <v>87</v>
       </c>
       <c r="J64">
@@ -4897,10 +4956,10 @@
       <c r="G65" s="9">
         <v>66.939583999999996</v>
       </c>
-      <c r="H65" s="69">
+      <c r="H65">
         <v>1593.5349120000001</v>
       </c>
-      <c r="I65" s="71" t="s">
+      <c r="I65" s="21" t="s">
         <v>86</v>
       </c>
       <c r="J65">
@@ -4932,10 +4991,10 @@
       <c r="G66" s="9">
         <v>66.939254000000005</v>
       </c>
-      <c r="H66" s="69">
+      <c r="H66">
         <v>1593.405884</v>
       </c>
-      <c r="I66" s="71" t="s">
+      <c r="I66" s="21" t="s">
         <v>85</v>
       </c>
       <c r="J66">
@@ -4967,10 +5026,10 @@
       <c r="G67" s="9">
         <v>66.938821000000004</v>
       </c>
-      <c r="H67" s="69">
+      <c r="H67">
         <v>1592.6748050000001</v>
       </c>
-      <c r="I67" s="71" t="s">
+      <c r="I67" s="21" t="s">
         <v>84</v>
       </c>
       <c r="J67">
@@ -5002,10 +5061,10 @@
       <c r="G68" s="9">
         <v>66.938365000000005</v>
       </c>
-      <c r="H68" s="69">
+      <c r="H68">
         <v>1592.3756100000001</v>
       </c>
-      <c r="I68" s="71" t="s">
+      <c r="I68" s="21" t="s">
         <v>83</v>
       </c>
       <c r="J68">
@@ -5037,10 +5096,10 @@
       <c r="G69" s="9">
         <v>66.937944000000002</v>
       </c>
-      <c r="H69" s="69">
+      <c r="H69">
         <v>1591.8110349999999</v>
       </c>
-      <c r="I69" s="71" t="s">
+      <c r="I69" s="21" t="s">
         <v>82</v>
       </c>
       <c r="J69">
@@ -5072,10 +5131,10 @@
       <c r="G70" s="9">
         <v>66.937631999999994</v>
       </c>
-      <c r="H70" s="69">
+      <c r="H70">
         <v>1591.160889</v>
       </c>
-      <c r="I70" s="71" t="s">
+      <c r="I70" s="21" t="s">
         <v>81</v>
       </c>
       <c r="J70">
@@ -5107,10 +5166,10 @@
       <c r="G71" s="9">
         <v>66.937146999999996</v>
       </c>
-      <c r="H71" s="69">
+      <c r="H71">
         <v>1590.496582</v>
       </c>
-      <c r="I71" s="71" t="s">
+      <c r="I71" s="21" t="s">
         <v>80</v>
       </c>
       <c r="J71">
@@ -5142,10 +5201,10 @@
       <c r="G72" s="9">
         <v>66.936881999999997</v>
       </c>
-      <c r="H72" s="69">
+      <c r="H72">
         <v>1589.931274</v>
       </c>
-      <c r="I72" s="71" t="s">
+      <c r="I72" s="21" t="s">
         <v>79</v>
       </c>
       <c r="J72">
@@ -5177,10 +5236,10 @@
       <c r="G73" s="9">
         <v>66.937048000000004</v>
       </c>
-      <c r="H73" s="69">
+      <c r="H73">
         <v>1590.084961</v>
       </c>
-      <c r="I73" s="71" t="s">
+      <c r="I73" s="21" t="s">
         <v>78</v>
       </c>
       <c r="J73">
@@ -5212,10 +5271,10 @@
       <c r="G74" s="9">
         <v>66.937054000000003</v>
       </c>
-      <c r="H74" s="69">
+      <c r="H74">
         <v>1590.036499</v>
       </c>
-      <c r="I74" s="71" t="s">
+      <c r="I74" s="21" t="s">
         <v>77</v>
       </c>
       <c r="J74">
@@ -5247,10 +5306,10 @@
       <c r="G75" s="9">
         <v>66.937258</v>
       </c>
-      <c r="H75" s="69">
+      <c r="H75">
         <v>1589.572876</v>
       </c>
-      <c r="I75" s="71" t="s">
+      <c r="I75" s="21" t="s">
         <v>76</v>
       </c>
       <c r="J75">
@@ -5282,10 +5341,10 @@
       <c r="G76" s="9">
         <v>66.937428999999995</v>
       </c>
-      <c r="H76" s="69">
+      <c r="H76">
         <v>1589.8602289999999</v>
       </c>
-      <c r="I76" s="71" t="s">
+      <c r="I76" s="21" t="s">
         <v>75</v>
       </c>
       <c r="J76">
@@ -5317,10 +5376,10 @@
       <c r="G77" s="9">
         <v>66.940203999999994</v>
       </c>
-      <c r="H77" s="69">
+      <c r="H77">
         <v>1591.2626949999999</v>
       </c>
-      <c r="I77" s="71" t="s">
+      <c r="I77" s="21" t="s">
         <v>74</v>
       </c>
       <c r="J77">
@@ -5352,10 +5411,10 @@
       <c r="G78" s="9">
         <v>66.940378999999993</v>
       </c>
-      <c r="H78" s="69">
+      <c r="H78">
         <v>1590.7044679999999</v>
       </c>
-      <c r="I78" s="71" t="s">
+      <c r="I78" s="21" t="s">
         <v>73</v>
       </c>
       <c r="J78">
@@ -5387,10 +5446,10 @@
       <c r="G79" s="9">
         <v>66.940735000000004</v>
       </c>
-      <c r="H79" s="69">
+      <c r="H79">
         <v>1590.493774</v>
       </c>
-      <c r="I79" s="71" t="s">
+      <c r="I79" s="21" t="s">
         <v>72</v>
       </c>
       <c r="J79">
@@ -5422,10 +5481,10 @@
       <c r="G80" s="9">
         <v>66.940924999999993</v>
       </c>
-      <c r="H80" s="69">
+      <c r="H80">
         <v>1589.6635739999999</v>
       </c>
-      <c r="I80" s="71" t="s">
+      <c r="I80" s="21" t="s">
         <v>71</v>
       </c>
       <c r="J80">
@@ -5457,10 +5516,10 @@
       <c r="G81" s="9">
         <v>66.941117000000006</v>
       </c>
-      <c r="H81" s="69">
+      <c r="H81">
         <v>1589.3792719999999</v>
       </c>
-      <c r="I81" s="71" t="s">
+      <c r="I81" s="21" t="s">
         <v>70</v>
       </c>
       <c r="J81">
@@ -5492,10 +5551,10 @@
       <c r="G82" s="9">
         <v>66.941140000000004</v>
       </c>
-      <c r="H82" s="69">
+      <c r="H82">
         <v>1589.345581</v>
       </c>
-      <c r="I82" s="71" t="s">
+      <c r="I82" s="21" t="s">
         <v>69</v>
       </c>
       <c r="J82">
@@ -5527,10 +5586,10 @@
       <c r="G83" s="9">
         <v>66.941145000000006</v>
       </c>
-      <c r="H83" s="69">
+      <c r="H83">
         <v>1589.306519</v>
       </c>
-      <c r="I83" s="71" t="s">
+      <c r="I83" s="21" t="s">
         <v>68</v>
       </c>
       <c r="J83">
@@ -5562,10 +5621,10 @@
       <c r="G84" s="9">
         <v>66.941036999999994</v>
       </c>
-      <c r="H84" s="69">
+      <c r="H84">
         <v>1588.945557</v>
       </c>
-      <c r="I84" s="71" t="s">
+      <c r="I84" s="21" t="s">
         <v>67</v>
       </c>
       <c r="J84">
@@ -5597,10 +5656,10 @@
       <c r="G85" s="9">
         <v>66.941417999999999</v>
       </c>
-      <c r="H85" s="69">
+      <c r="H85">
         <v>1589.2055660000001</v>
       </c>
-      <c r="I85" s="71" t="s">
+      <c r="I85" s="21" t="s">
         <v>66</v>
       </c>
       <c r="J85">
@@ -5632,10 +5691,10 @@
       <c r="G86" s="9">
         <v>66.941922000000005</v>
       </c>
-      <c r="H86" s="69">
+      <c r="H86">
         <v>1589.2734379999999</v>
       </c>
-      <c r="I86" s="71" t="s">
+      <c r="I86" s="21" t="s">
         <v>65</v>
       </c>
       <c r="J86">
@@ -5667,10 +5726,10 @@
       <c r="G87" s="9">
         <v>66.942234999999997</v>
       </c>
-      <c r="H87" s="69">
+      <c r="H87">
         <v>1589.8176269999999</v>
       </c>
-      <c r="I87" s="71" t="s">
+      <c r="I87" s="21" t="s">
         <v>64</v>
       </c>
       <c r="J87">
@@ -5702,10 +5761,10 @@
       <c r="G88" s="9">
         <v>66.942559000000003</v>
       </c>
-      <c r="H88" s="69">
+      <c r="H88">
         <v>1589.3055420000001</v>
       </c>
-      <c r="I88" s="71" t="s">
+      <c r="I88" s="21" t="s">
         <v>63</v>
       </c>
       <c r="J88">
@@ -5737,10 +5796,10 @@
       <c r="G89" s="9">
         <v>66.942882999999995</v>
       </c>
-      <c r="H89" s="69">
+      <c r="H89">
         <v>1589.5466309999999</v>
       </c>
-      <c r="I89" s="71" t="s">
+      <c r="I89" s="21" t="s">
         <v>62</v>
       </c>
       <c r="J89">
@@ -5772,10 +5831,10 @@
       <c r="G90" s="9">
         <v>66.943325999999999</v>
       </c>
-      <c r="H90" s="69">
+      <c r="H90">
         <v>1589.6695560000001</v>
       </c>
-      <c r="I90" s="71" t="s">
+      <c r="I90" s="21" t="s">
         <v>61</v>
       </c>
       <c r="J90">
@@ -5807,10 +5866,10 @@
       <c r="G91" s="9">
         <v>66.943297999999999</v>
       </c>
-      <c r="H91" s="69">
+      <c r="H91">
         <v>1594.4554439999999</v>
       </c>
-      <c r="I91" s="71" t="s">
+      <c r="I91" s="21" t="s">
         <v>60</v>
       </c>
       <c r="J91">
@@ -5842,10 +5901,10 @@
       <c r="G92" s="9">
         <v>66.943315999999996</v>
       </c>
-      <c r="H92" s="69">
+      <c r="H92">
         <v>1594.3551030000001</v>
       </c>
-      <c r="I92" s="71" t="s">
+      <c r="I92" s="21" t="s">
         <v>59</v>
       </c>
       <c r="J92">
@@ -5877,10 +5936,10 @@
       <c r="G93" s="9">
         <v>66.943433999999996</v>
       </c>
-      <c r="H93" s="69">
+      <c r="H93">
         <v>1598.679932</v>
       </c>
-      <c r="I93" s="71" t="s">
+      <c r="I93" s="21" t="s">
         <v>54</v>
       </c>
       <c r="J93">
@@ -5986,8 +6045,9 @@
     <hyperlink ref="C93" r:id="rId92" xr:uid="{B4E89D93-459F-4C87-AB6F-C3C3B7AF1670}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId93"/>
   <tableParts count="1">
-    <tablePart r:id="rId93"/>
+    <tablePart r:id="rId94"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6004,12 +6064,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.5">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="78" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="12" t="s">

</xml_diff>